<commit_message>
READY: 5 parsers connected with server
</commit_message>
<xml_diff>
--- a/init_uploads/download_files/Копия Список поставщиков.xlsx
+++ b/init_uploads/download_files/Копия Список поставщиков.xlsx
@@ -70,7 +70,7 @@
     <t xml:space="preserve">Холод-Климат Сма</t>
   </si>
   <si>
-    <t xml:space="preserve">Uriarte taldea</t>
+    <t xml:space="preserve">Uriarte</t>
   </si>
   <si>
     <t xml:space="preserve">Favale</t>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Torrington</t>
   </si>
   <si>
-    <t xml:space="preserve">Fluorgas Necton</t>
+    <t xml:space="preserve">Fluorgaz</t>
   </si>
   <si>
     <t xml:space="preserve">Климат</t>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">https://www.fijamom.com.ar/</t>
   </si>
   <si>
-    <t xml:space="preserve">Distribuidora Belgrano</t>
+    <t xml:space="preserve">Belgrano</t>
   </si>
   <si>
     <t xml:space="preserve">https://catalogo.duxsoftware.com.ar/3820</t>

</xml_diff>

<commit_message>
READY: web-parsers connected with server
</commit_message>
<xml_diff>
--- a/init_uploads/download_files/Копия Список поставщиков.xlsx
+++ b/init_uploads/download_files/Копия Список поставщиков.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="83">
   <si>
     <t xml:space="preserve">Рубрика</t>
   </si>
@@ -73,7 +73,13 @@
     <t xml:space="preserve">Uriarte</t>
   </si>
   <si>
+    <t xml:space="preserve">https://uriarte.com.ar/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Favale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.repuestosfavale.com/</t>
   </si>
   <si>
     <t xml:space="preserve">Фреон</t>
@@ -82,7 +88,13 @@
     <t xml:space="preserve">Torrington</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.torrington.com.ar/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fluorgaz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://listado.mercadolibre.com.ar/fluor-gas-refrigerantes</t>
   </si>
   <si>
     <t xml:space="preserve">Климат</t>
@@ -115,13 +127,22 @@
     <t xml:space="preserve">Electrofrig</t>
   </si>
   <si>
+    <t xml:space="preserve">http://www.electrofrig.com.ar/es/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Electrocity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://electrocity.com.ar</t>
   </si>
   <si>
     <t xml:space="preserve">Масла</t>
   </si>
   <si>
     <t xml:space="preserve">Refrioil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://refrioil.com/</t>
   </si>
   <si>
     <t xml:space="preserve">Тэн холодильника</t>
@@ -136,6 +157,9 @@
     <t xml:space="preserve">IMI</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.instagram.com/imi.metalurgica.integral/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Сма</t>
   </si>
   <si>
@@ -145,7 +169,13 @@
     <t xml:space="preserve">Roma Repuestos insumos</t>
   </si>
   <si>
+    <t xml:space="preserve">https://tienda.romarep.com.ar/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oeste service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://oesteservice.com.ar/</t>
   </si>
   <si>
     <t xml:space="preserve">Distribuidora JC</t>
@@ -166,7 +196,13 @@
     <t xml:space="preserve">Dpmg Anton</t>
   </si>
   <si>
+    <t xml:space="preserve">https://www.dpmg.com.ar/brand/anton/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tidar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://tidar.com.ar/</t>
   </si>
   <si>
     <t xml:space="preserve">Casa Jarse</t>
@@ -178,10 +214,19 @@
     <t xml:space="preserve">Lujumar srl</t>
   </si>
   <si>
+    <t xml:space="preserve">https://lujumar.com.ar/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Norfrig</t>
   </si>
   <si>
+    <t xml:space="preserve">https://norfrig.com.ar/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pilisar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://pilisardistribuidor.com.ar/</t>
   </si>
   <si>
     <t xml:space="preserve">Подшипники</t>
@@ -193,10 +238,16 @@
     <t xml:space="preserve">Industrias MCT</t>
   </si>
   <si>
+    <t xml:space="preserve">https://industriasmct.com</t>
+  </si>
+  <si>
     <t xml:space="preserve">СВЧ</t>
   </si>
   <si>
     <t xml:space="preserve">Guillermo pini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://pini.com.ar/</t>
   </si>
   <si>
     <t xml:space="preserve">СВЧ и котлы</t>
@@ -205,10 +256,16 @@
     <t xml:space="preserve">Damfer</t>
   </si>
   <si>
+    <t xml:space="preserve">https://damfer.com/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Конденсаторы</t>
   </si>
   <si>
     <t xml:space="preserve">Persano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.persano.com.ar/index.php</t>
   </si>
   <si>
     <t xml:space="preserve">Итог по холоду и климату</t>
@@ -675,7 +732,10 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.43"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="3" style="1" width="10.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="4" min="4" style="1" width="14.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="6" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="8" style="1" width="8.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="1" width="10.16"/>
   </cols>
   <sheetData>
@@ -854,7 +914,9 @@
       <c r="D6" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -878,13 +940,15 @@
         <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" s="9"/>
       <c r="D7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="E7" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -905,16 +969,18 @@
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -935,16 +1001,18 @@
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -965,10 +1033,10 @@
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>9</v>
@@ -977,7 +1045,7 @@
         <v>9</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1002,7 +1070,7 @@
         <v>15</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>9</v>
@@ -1011,7 +1079,7 @@
         <v>9</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1033,10 +1101,10 @@
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>9</v>
@@ -1045,7 +1113,7 @@
         <v>9</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1067,16 +1135,18 @@
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -1098,11 +1168,13 @@
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="7"/>
-      <c r="E14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -1123,16 +1195,18 @@
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -1153,10 +1227,10 @@
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="7" t="s">
@@ -1183,16 +1257,18 @@
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -1213,10 +1289,10 @@
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="7" t="s">
@@ -1243,10 +1319,10 @@
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>9</v>
@@ -1254,7 +1330,9 @@
       <c r="D19" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -1275,16 +1353,18 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -1305,10 +1385,10 @@
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>9</v>
@@ -1317,7 +1397,7 @@
         <v>9</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1339,10 +1419,10 @@
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>9</v>
@@ -1351,7 +1431,7 @@
         <v>9</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1373,16 +1453,18 @@
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -1404,11 +1486,13 @@
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
       <c r="B24" s="12" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="7"/>
-      <c r="E24" s="2"/>
+      <c r="E24" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -1430,12 +1514,12 @@
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="7"/>
       <c r="E25" s="11" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1457,14 +1541,16 @@
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="7"/>
-      <c r="E26" s="2"/>
+      <c r="E26" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -1485,14 +1571,16 @@
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="E27" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -1513,14 +1601,16 @@
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>53</v>
+        <v>67</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="7"/>
-      <c r="E28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -1541,10 +1631,10 @@
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1570,11 +1660,13 @@
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>56</v>
+        <v>71</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="E30" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -1595,14 +1687,16 @@
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
+      <c r="E31" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1623,16 +1717,18 @@
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E32" s="2"/>
+      <c r="E32" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -1653,14 +1749,16 @@
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="E33" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -1681,7 +1779,7 @@
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>63</v>
+        <v>82</v>
       </c>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
@@ -24620,11 +24718,30 @@
     <hyperlink ref="E3" r:id="rId1" display="https://www.ansal.com.ar/"/>
     <hyperlink ref="E4" r:id="rId2" display="https://www.reld.com.ar/"/>
     <hyperlink ref="E5" r:id="rId3" display="www.bellinihnos.com.ar/"/>
-    <hyperlink ref="E10" r:id="rId4" display="https://www.fijamom.com.ar/"/>
-    <hyperlink ref="E11" r:id="rId5" display="https://catalogo.duxsoftware.com.ar/3820"/>
-    <hyperlink ref="E12" r:id="rId6" display="https://www.agrupacionduna.com/"/>
-    <hyperlink ref="E21" r:id="rId7" display="https://distribuidorajc.com/"/>
-    <hyperlink ref="E25" r:id="rId8" display="https://casajarse.com/"/>
+    <hyperlink ref="E6" r:id="rId4" display="https://uriarte.com.ar/"/>
+    <hyperlink ref="E7" r:id="rId5" display="https://www.repuestosfavale.com/"/>
+    <hyperlink ref="E8" r:id="rId6" display="https://www.torrington.com.ar/"/>
+    <hyperlink ref="E9" r:id="rId7" display="https://listado.mercadolibre.com.ar/fluor-gas-refrigerantes"/>
+    <hyperlink ref="E10" r:id="rId8" display="https://www.fijamom.com.ar/"/>
+    <hyperlink ref="E11" r:id="rId9" display="https://catalogo.duxsoftware.com.ar/3820"/>
+    <hyperlink ref="E12" r:id="rId10" display="https://www.agrupacionduna.com/"/>
+    <hyperlink ref="E13" r:id="rId11" display="http://www.electrofrig.com.ar/es/"/>
+    <hyperlink ref="E14" r:id="rId12" display="https://electrocity.com.ar"/>
+    <hyperlink ref="E15" r:id="rId13" display="https://refrioil.com/"/>
+    <hyperlink ref="E17" r:id="rId14" display="https://www.instagram.com/imi.metalurgica.integral/"/>
+    <hyperlink ref="E19" r:id="rId15" display="https://tienda.romarep.com.ar/"/>
+    <hyperlink ref="E20" r:id="rId16" display="https://oesteservice.com.ar/"/>
+    <hyperlink ref="E21" r:id="rId17" display="https://distribuidorajc.com/"/>
+    <hyperlink ref="E23" r:id="rId18" display="https://www.dpmg.com.ar/brand/anton/"/>
+    <hyperlink ref="E24" r:id="rId19" display="https://tidar.com.ar/"/>
+    <hyperlink ref="E25" r:id="rId20" display="https://casajarse.com/"/>
+    <hyperlink ref="E26" r:id="rId21" display="https://lujumar.com.ar/"/>
+    <hyperlink ref="E27" r:id="rId22" display="https://norfrig.com.ar/"/>
+    <hyperlink ref="E28" r:id="rId23" display="https://pilisardistribuidor.com.ar/"/>
+    <hyperlink ref="E30" r:id="rId24" display="https://industriasmct.com"/>
+    <hyperlink ref="E31" r:id="rId25" display="https://pini.com.ar/"/>
+    <hyperlink ref="E32" r:id="rId26" display="https://damfer.com/"/>
+    <hyperlink ref="E33" r:id="rId27" display="https://www.persano.com.ar/index.php"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
final price added to productsupplier
</commit_message>
<xml_diff>
--- a/init_uploads/download_files/Копия Список поставщиков.xlsx
+++ b/init_uploads/download_files/Копия Список поставщиков.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="85">
   <si>
     <t xml:space="preserve">Рубрика</t>
   </si>
@@ -41,6 +41,12 @@
   </si>
   <si>
     <t xml:space="preserve">Пароль</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Скидка %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA</t>
   </si>
   <si>
     <t xml:space="preserve">Холод-Климат</t>
@@ -275,8 +281,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -415,7 +422,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -449,6 +456,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -732,10 +743,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.43"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="3" min="3" style="1" width="10.29"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="4" min="4" style="1" width="14.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="8" style="1" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="9" style="1" width="8.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="1" width="10.16"/>
   </cols>
   <sheetData>
@@ -785,8 +797,12 @@
       <c r="G2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
@@ -803,24 +819,28 @@
     </row>
     <row r="3" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="9" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
@@ -837,19 +857,19 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>9</v>
-      </c>
       <c r="D4" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -871,19 +891,19 @@
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -905,17 +925,17 @@
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
-      <c r="C6" s="9"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -937,17 +957,17 @@
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
-      <c r="C7" s="9"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -969,17 +989,17 @@
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1001,17 +1021,17 @@
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1033,19 +1053,19 @@
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>27</v>
+      <c r="E10" s="11" t="s">
+        <v>29</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1067,19 +1087,19 @@
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
-      <c r="E11" s="11" t="s">
-        <v>29</v>
+      <c r="E11" s="12" t="s">
+        <v>31</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1101,19 +1121,19 @@
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1135,17 +1155,17 @@
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1168,12 +1188,12 @@
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="7"/>
       <c r="E14" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1195,17 +1215,17 @@
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1227,14 +1247,14 @@
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -1257,17 +1277,17 @@
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1289,14 +1309,14 @@
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -1319,19 +1339,19 @@
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1353,17 +1373,17 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1385,19 +1405,19 @@
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
-      <c r="E21" s="10" t="s">
-        <v>53</v>
+      <c r="E21" s="11" t="s">
+        <v>55</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1419,19 +1439,19 @@
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1453,17 +1473,17 @@
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
-      <c r="C23" s="9"/>
+      <c r="C23" s="10"/>
       <c r="D23" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1485,13 +1505,13 @@
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
-      <c r="B24" s="12" t="s">
-        <v>59</v>
+      <c r="B24" s="13" t="s">
+        <v>61</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="7"/>
       <c r="E24" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1514,12 +1534,12 @@
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="7"/>
-      <c r="E25" s="11" t="s">
-        <v>62</v>
+      <c r="E25" s="12" t="s">
+        <v>64</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1541,15 +1561,15 @@
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="7"/>
       <c r="E26" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1571,15 +1591,15 @@
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1601,15 +1621,15 @@
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="7"/>
       <c r="E28" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1631,10 +1651,10 @@
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1660,12 +1680,12 @@
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1687,15 +1707,15 @@
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1717,17 +1737,17 @@
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1749,15 +1769,15 @@
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -1778,12 +1798,12 @@
       <c r="V33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>82</v>
+      <c r="A34" s="14" t="s">
+        <v>84</v>
       </c>
-      <c r="B34" s="13"/>
-      <c r="C34" s="13"/>
-      <c r="D34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="15"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>

</xml_diff>

<commit_message>
READY: initial Celery-Redis refactoring
</commit_message>
<xml_diff>
--- a/init_uploads/download_files/Копия Список поставщиков.xlsx
+++ b/init_uploads/download_files/Копия Список поставщиков.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="95">
   <si>
     <t xml:space="preserve">Рубрика</t>
   </si>
@@ -73,6 +73,9 @@
     <t xml:space="preserve">https://www.reld.com.ar/</t>
   </si>
   <si>
+    <t xml:space="preserve">Reld%2024foT</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bellini</t>
   </si>
   <si>
@@ -121,6 +124,12 @@
     <t xml:space="preserve">https://www.fijamom.com.ar/</t>
   </si>
   <si>
+    <t xml:space="preserve">dashamalkina.sf@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sbtinternational</t>
+  </si>
+  <si>
     <t xml:space="preserve">Belgrano</t>
   </si>
   <si>
@@ -136,6 +145,12 @@
     <t xml:space="preserve">https://www.agrupacionduna.com/</t>
   </si>
   <si>
+    <t xml:space="preserve">sbt.international.srl@gmail.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asdfghjkl2024</t>
+  </si>
+  <si>
     <t xml:space="preserve">Компресора</t>
   </si>
   <si>
@@ -145,10 +160,16 @@
     <t xml:space="preserve">http://www.electrofrig.com.ar/es/</t>
   </si>
   <si>
+    <t xml:space="preserve">Asdfghj-2025</t>
+  </si>
+  <si>
     <t xml:space="preserve">Electrocity</t>
   </si>
   <si>
     <t xml:space="preserve">https://electrocity.com.ar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sbtint2026</t>
   </si>
   <si>
     <t xml:space="preserve">Масла</t>
@@ -846,8 +867,12 @@
       <c r="E3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" s="2" t="n">
+        <v>254902</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>30718398254</v>
+      </c>
       <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
@@ -887,8 +912,12 @@
       <c r="E4" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="2" t="n">
+        <v>30718398254</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="H4" s="2" t="s">
         <v>14</v>
       </c>
@@ -913,7 +942,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>12</v>
@@ -922,7 +951,7 @@
         <v>12</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -947,22 +976,22 @@
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -982,17 +1011,17 @@
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1017,17 +1046,17 @@
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1052,22 +1081,22 @@
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -1087,10 +1116,10 @@
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>12</v>
@@ -1099,10 +1128,14 @@
         <v>12</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="H10" s="2" t="s">
         <v>14</v>
       </c>
@@ -1124,10 +1157,10 @@
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>12</v>
@@ -1136,7 +1169,7 @@
         <v>12</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1161,10 +1194,10 @@
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>12</v>
@@ -1173,10 +1206,14 @@
         <v>12</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>14</v>
       </c>
@@ -1198,22 +1235,26 @@
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="F13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="H13" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
@@ -1234,15 +1275,19 @@
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="2"/>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="7"/>
       <c r="E14" s="2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="H14" s="2" t="s">
         <v>14</v>
       </c>
@@ -1264,17 +1309,17 @@
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1299,10 +1344,10 @@
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="7" t="s">
@@ -1332,17 +1377,17 @@
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1367,10 +1412,10 @@
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="7" t="s">
@@ -1400,10 +1445,10 @@
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>12</v>
@@ -1412,10 +1457,14 @@
         <v>12</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="F19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>12345678</v>
+      </c>
       <c r="H19" s="2" t="s">
         <v>14</v>
       </c>
@@ -1437,17 +1486,17 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1472,10 +1521,10 @@
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>12</v>
@@ -1484,7 +1533,7 @@
         <v>12</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1509,10 +1558,10 @@
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>12</v>
@@ -1521,7 +1570,7 @@
         <v>12</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1546,17 +1595,17 @@
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1582,12 +1631,12 @@
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2"/>
       <c r="B24" s="13" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="7"/>
       <c r="E24" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1613,12 +1662,12 @@
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="7"/>
       <c r="E25" s="12" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1643,15 +1692,15 @@
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="7"/>
       <c r="E26" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1676,18 +1725,22 @@
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="F27" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="H27" s="2" t="s">
         <v>14</v>
       </c>
@@ -1709,15 +1762,15 @@
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="7"/>
       <c r="E28" s="2" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1742,10 +1795,10 @@
     </row>
     <row r="29" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1774,12 +1827,12 @@
     <row r="30" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1804,15 +1857,15 @@
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1837,17 +1890,17 @@
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="7" t="s">
         <v>12</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1872,15 +1925,15 @@
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -1905,7 +1958,7 @@
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
@@ -25804,25 +25857,31 @@
     <hyperlink ref="E8" r:id="rId6" display="https://www.torrington.com.ar/"/>
     <hyperlink ref="E9" r:id="rId7" display="https://listado.mercadolibre.com.ar/fluor-gas-refrigerantes"/>
     <hyperlink ref="E10" r:id="rId8" display="https://www.fijamom.com.ar/"/>
-    <hyperlink ref="E11" r:id="rId9" display="https://catalogo.duxsoftware.com.ar/3820"/>
-    <hyperlink ref="E12" r:id="rId10" display="https://www.agrupacionduna.com/"/>
-    <hyperlink ref="E13" r:id="rId11" display="http://www.electrofrig.com.ar/es/"/>
-    <hyperlink ref="E14" r:id="rId12" display="https://electrocity.com.ar"/>
-    <hyperlink ref="E15" r:id="rId13" display="https://refrioil.com/"/>
-    <hyperlink ref="E17" r:id="rId14" display="https://www.instagram.com/imi.metalurgica.integral/"/>
-    <hyperlink ref="E19" r:id="rId15" display="https://tienda.romarep.com.ar/"/>
-    <hyperlink ref="E20" r:id="rId16" display="https://oesteservice.com.ar/"/>
-    <hyperlink ref="E21" r:id="rId17" display="https://distribuidorajc.com/"/>
-    <hyperlink ref="E23" r:id="rId18" display="https://www.dpmg.com.ar/brand/anton/"/>
-    <hyperlink ref="E24" r:id="rId19" display="https://tidar.com.ar/"/>
-    <hyperlink ref="E25" r:id="rId20" display="https://casajarse.com/"/>
-    <hyperlink ref="E26" r:id="rId21" display="https://lujumar.com.ar/"/>
-    <hyperlink ref="E27" r:id="rId22" display="https://norfrig.com.ar/"/>
-    <hyperlink ref="E28" r:id="rId23" display="https://pilisardistribuidor.com.ar/"/>
-    <hyperlink ref="E30" r:id="rId24" display="https://industriasmct.com"/>
-    <hyperlink ref="E31" r:id="rId25" display="https://pini.com.ar/"/>
-    <hyperlink ref="E32" r:id="rId26" display="https://damfer.com/"/>
-    <hyperlink ref="E33" r:id="rId27" display="https://www.persano.com.ar/index.php"/>
+    <hyperlink ref="F10" r:id="rId9" display="dashamalkina.sf@gmail.com"/>
+    <hyperlink ref="E11" r:id="rId10" display="https://catalogo.duxsoftware.com.ar/3820"/>
+    <hyperlink ref="E12" r:id="rId11" display="https://www.agrupacionduna.com/"/>
+    <hyperlink ref="F12" r:id="rId12" display="sbt.international.srl@gmail.com"/>
+    <hyperlink ref="E13" r:id="rId13" display="http://www.electrofrig.com.ar/es/"/>
+    <hyperlink ref="F13" r:id="rId14" display="sbt.international.srl@gmail.com"/>
+    <hyperlink ref="E14" r:id="rId15" display="https://electrocity.com.ar"/>
+    <hyperlink ref="F14" r:id="rId16" display="sbt.international.srl@gmail.com"/>
+    <hyperlink ref="E15" r:id="rId17" display="https://refrioil.com/"/>
+    <hyperlink ref="E17" r:id="rId18" display="https://www.instagram.com/imi.metalurgica.integral/"/>
+    <hyperlink ref="E19" r:id="rId19" display="https://tienda.romarep.com.ar/"/>
+    <hyperlink ref="F19" r:id="rId20" display="sbt.international.srl@gmail.com"/>
+    <hyperlink ref="E20" r:id="rId21" display="https://oesteservice.com.ar/"/>
+    <hyperlink ref="E21" r:id="rId22" display="https://distribuidorajc.com/"/>
+    <hyperlink ref="E23" r:id="rId23" display="https://www.dpmg.com.ar/brand/anton/"/>
+    <hyperlink ref="E24" r:id="rId24" display="https://tidar.com.ar/"/>
+    <hyperlink ref="E25" r:id="rId25" display="https://casajarse.com/"/>
+    <hyperlink ref="E26" r:id="rId26" display="https://lujumar.com.ar/"/>
+    <hyperlink ref="E27" r:id="rId27" display="https://norfrig.com.ar/"/>
+    <hyperlink ref="F27" r:id="rId28" display="sbt.international.srl@gmail.com"/>
+    <hyperlink ref="E28" r:id="rId29" display="https://pilisardistribuidor.com.ar/"/>
+    <hyperlink ref="E30" r:id="rId30" display="https://industriasmct.com"/>
+    <hyperlink ref="E31" r:id="rId31" display="https://pini.com.ar/"/>
+    <hyperlink ref="E32" r:id="rId32" display="https://damfer.com/"/>
+    <hyperlink ref="E33" r:id="rId33" display="https://www.persano.com.ar/index.php"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>